<commit_message>
update onboarding and maintainence flow
</commit_message>
<xml_diff>
--- a/frontend-web/public/templates/SLMS2026_import_tenant_draft_contracts.xlsx
+++ b/frontend-web/public/templates/SLMS2026_import_tenant_draft_contracts.xlsx
@@ -573,7 +573,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:S6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -610,24 +610,27 @@
         <v>Nơi cấp CCCD</v>
       </c>
       <c r="L1" t="str">
+        <v>Hộ khẩu thường trú</v>
+      </c>
+      <c r="M1" t="str">
         <v>Ngày vào ở</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Ngày kết thúc</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Giá thuê/tháng</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Số tháng cọc</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Tiền cọc</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Ngày đón khách dự kiến</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>SĐT quản lý đón khách</v>
       </c>
     </row>
@@ -666,24 +669,27 @@
         <v>CA TP. Hồ Chí Minh</v>
       </c>
       <c r="L2" t="str">
+        <v>123 Nguyễn Huệ, Q1, TP.HCM</v>
+      </c>
+      <c r="M2" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>2027-07-31</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>8000000</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>1</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>8000000</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
         <v/>
       </c>
     </row>
@@ -722,24 +728,27 @@
         <v>CA Quận 1</v>
       </c>
       <c r="L3" t="str">
+        <v>45 Lê Lợi, Q1, TP.HCM</v>
+      </c>
+      <c r="M3" t="str">
         <v>01/09/2026</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>31/08/2027</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>9500000</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>2</v>
       </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
       <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
         <v>01/09/2026</v>
       </c>
-      <c r="R3" t="str">
+      <c r="S3" t="str">
         <v/>
       </c>
     </row>
@@ -778,24 +787,27 @@
         <v>CA Bình Thạnh</v>
       </c>
       <c r="L4" t="str">
+        <v>88 Phạm Văn Đồng, Bình Thạnh, TP.HCM</v>
+      </c>
+      <c r="M4" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>2027-08-14</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>4500000</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>1</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>4500000</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
         <v/>
       </c>
     </row>
@@ -834,24 +846,27 @@
         <v>CA Gò Vấp</v>
       </c>
       <c r="L5" t="str">
+        <v>12 Quang Trung, Gò Vấp, TP.HCM</v>
+      </c>
+      <c r="M5" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>2027-02-14</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>4200000</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>1</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>4200000</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="R5" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="R5" t="str">
+      <c r="S5" t="str">
         <v/>
       </c>
     </row>
@@ -890,30 +905,33 @@
         <v>CA Phú Nhuận</v>
       </c>
       <c r="L6" t="str">
+        <v>56 Nguyễn Văn Trỗi, Phú Nhuận, TP.HCM</v>
+      </c>
+      <c r="M6" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>2027-08-31</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>5000000</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>2</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>10000000</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="R6" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="R6" t="str">
+      <c r="S6" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add zone assignment/import features and update tenant onboarding flow
- Add manager-zone assignment page and Excel import wizard for zones (frontend-web)
- Update draft contract form, import modal, and onboarding list to reflect operationManagerId-driven assignment
- Update contract monitoring, zone management/form modal, tenant/zone services and API types accordingly
- Update mobile-app onboarding, contract, and maintenance screens/services to match; remove dead MeterReadingScreen
- Prepare Vercel deployment config: vercel.json SPA rewrite, VITE_API_URL-based axios baseURL with 90s timeout for Render cold start, error field priority fix
</commit_message>
<xml_diff>
--- a/frontend-web/public/templates/SLMS2026_import_tenant_draft_contracts.xlsx
+++ b/frontend-web/public/templates/SLMS2026_import_tenant_draft_contracts.xlsx
@@ -573,7 +573,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:R6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -630,9 +630,6 @@
       <c r="R1" t="str">
         <v>Ngày đón khách dự kiến</v>
       </c>
-      <c r="S1" t="str">
-        <v>SĐT quản lý đón khách</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -689,9 +686,6 @@
       <c r="R2" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -748,9 +742,6 @@
       <c r="R3" t="str">
         <v>01/09/2026</v>
       </c>
-      <c r="S3" t="str">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -807,9 +798,6 @@
       <c r="R4" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="S4" t="str">
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -866,9 +854,6 @@
       <c r="R5" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="S5" t="str">
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -925,13 +910,10 @@
       <c r="R6" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="S6" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>